<commit_message>
mise en forme du tableau , premier jet
</commit_message>
<xml_diff>
--- a/Tab_Competence.xlsx
+++ b/Tab_Competence.xlsx
@@ -1,17 +1,26 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
   <workbookPr/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\elpek\Desktop\Project_Folder\projetisimag6\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A1EC949D-40DB-4F22-BDC1-C7650D9DB573}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <bookViews>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+  </bookViews>
   <sheets>
-    <sheet state="visible" name="Feuille 1" sheetId="1" r:id="rId5"/>
+    <sheet name="Feuille 1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <definedNames/>
-  <calcPr/>
+  <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="28" uniqueCount="28">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="54" uniqueCount="34">
   <si>
     <t>l1.1</t>
   </si>
@@ -88,33 +97,53 @@
     <t>COMMENTS</t>
   </si>
   <si>
-    <t>Issam</t>
-  </si>
-  <si>
     <t>Nabil</t>
   </si>
   <si>
     <t>Gahui</t>
+  </si>
+  <si>
+    <t>I</t>
+  </si>
+  <si>
+    <t>X</t>
+  </si>
+  <si>
+    <t>DFSP</t>
+  </si>
+  <si>
+    <t>B</t>
+  </si>
+  <si>
+    <t>phase préliminaire du projet, peu d'aspect envisagé, à corriger au plus vite</t>
+  </si>
+  <si>
+    <t>Eleves</t>
+  </si>
+  <si>
+    <t>BEN AHMED Issam</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-  <fonts count="3">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
-      <sz val="10.0"/>
+      <sz val="10"/>
       <color rgb="FF000000"/>
       <name val="Arial"/>
       <scheme val="minor"/>
     </font>
     <font>
+      <sz val="10"/>
       <color theme="1"/>
       <name val="Arial"/>
       <scheme val="minor"/>
     </font>
     <font>
       <b/>
+      <sz val="10"/>
       <color rgb="FFFF0000"/>
       <name val="Arial"/>
       <scheme val="minor"/>
@@ -125,43 +154,114 @@
       <patternFill patternType="none"/>
     </fill>
     <fill>
-      <patternFill patternType="lightGray"/>
+      <patternFill patternType="gray125"/>
     </fill>
   </fills>
   <borders count="1">
-    <border/>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
-    <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
   <cellXfs count="3">
-    <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0"/>
-    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle xfId="0" name="Normal" builtinId="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="0"/>
+  <dxfs count="2">
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="10"/>
+        <color theme="1"/>
+        <name val="Arial"/>
+        <scheme val="minor"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="10"/>
+        <color theme="1"/>
+        <name val="Arial"/>
+        <scheme val="minor"/>
+      </font>
+    </dxf>
+  </dxfs>
+  <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
 </file>
 
-<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
-<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:cx="http://schemas.microsoft.com/office/drawing/2014/chartex" xmlns:cx1="http://schemas.microsoft.com/office/drawing/2015/9/8/chartex" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:dgm="http://schemas.openxmlformats.org/drawingml/2006/diagram" xmlns:x3Unk="http://schemas.microsoft.com/office/drawing/2010/slicer" xmlns:sle15="http://schemas.microsoft.com/office/drawing/2012/slicer"/>
-</file>
-
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<x18tc:personList xmlns:x18tc="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments"/>
+<file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{8CF6DF7F-EEF8-49C3-8A48-08F5489EA84E}" name="Tableau1" displayName="Tableau1" ref="A1:Z4" totalsRowShown="0" headerRowDxfId="0">
+  <autoFilter ref="A1:Z4" xr:uid="{8CF6DF7F-EEF8-49C3-8A48-08F5489EA84E}"/>
+  <tableColumns count="26">
+    <tableColumn id="1" xr3:uid="{80165D86-5FBE-462D-9010-480F62D044FD}" name="Eleves" dataDxfId="1"/>
+    <tableColumn id="2" xr3:uid="{11E9BDD4-3F0D-4426-B9F2-AFFD5B6117DA}" name="l1.1"/>
+    <tableColumn id="3" xr3:uid="{53392726-0C02-454A-A689-6C9C69DCB944}" name="l1.2"/>
+    <tableColumn id="4" xr3:uid="{0D6EDA59-7CBD-47E8-B979-344526AFCB68}" name="l1.3"/>
+    <tableColumn id="5" xr3:uid="{6E346867-CE33-4DBB-846A-7C6C7638169B}" name="l1.4"/>
+    <tableColumn id="6" xr3:uid="{4251C954-C76C-4948-9C4E-BEFC327DF8D6}" name="l1.5"/>
+    <tableColumn id="7" xr3:uid="{E433E890-1939-420E-AEB4-7D222764C4B8}" name="l1.6"/>
+    <tableColumn id="8" xr3:uid="{E5F5157A-CC01-4A22-BA7D-D0F4E0B499B5}" name="l2.1"/>
+    <tableColumn id="9" xr3:uid="{7F5D1AD8-747B-411D-8A48-287530F84B4E}" name="l2.2"/>
+    <tableColumn id="10" xr3:uid="{68C79406-4D1A-47BF-8CD1-4C4C168E1791}" name="l2.3"/>
+    <tableColumn id="11" xr3:uid="{86F3AF26-A0E7-4BFE-B288-E8224142DF3A}" name="l2.4"/>
+    <tableColumn id="12" xr3:uid="{264ADEB2-9C16-4ACE-ABF1-1833A5234D4C}" name="l2.5"/>
+    <tableColumn id="13" xr3:uid="{E26FC957-CE4D-4AAF-B62B-C4EB16B3C611}" name="l2.6"/>
+    <tableColumn id="14" xr3:uid="{B8DADC49-D782-4960-87E9-BDFA8F8409AF}" name="l3.1"/>
+    <tableColumn id="15" xr3:uid="{017BBC1B-0C6E-4818-8A29-949F61AEA567}" name="l3.2"/>
+    <tableColumn id="16" xr3:uid="{4E4B0303-4617-478E-9639-ECBEABC7590F}" name="l3.3"/>
+    <tableColumn id="17" xr3:uid="{91B456CD-CD68-4E8A-87F4-647146366362}" name="l3.4"/>
+    <tableColumn id="18" xr3:uid="{17B3BF90-10AB-4E97-A867-CFFCE5A25966}" name="l3.5"/>
+    <tableColumn id="19" xr3:uid="{83C8DAB9-CEFC-40F2-BC9D-73129C0CE966}" name="l3.6"/>
+    <tableColumn id="20" xr3:uid="{64BD589A-A976-4984-B094-A4762EEEE028}" name="l3.7"/>
+    <tableColumn id="21" xr3:uid="{078F14D4-CC89-4041-87AA-8470B1F82BC3}" name="l4.1"/>
+    <tableColumn id="22" xr3:uid="{2934E05C-87F7-4DA8-B52F-569A7C24F9BB}" name="l4.2"/>
+    <tableColumn id="23" xr3:uid="{97166823-B29B-4057-BA3C-1CDB868E42A2}" name="l4.3"/>
+    <tableColumn id="24" xr3:uid="{9FF3D136-6898-42E9-9EB7-6BBBA4E8FA0A}" name="l4.4"/>
+    <tableColumn id="25" xr3:uid="{033EE8BA-A5AE-47D5-907F-881FA1A4065C}" name="l4.5"/>
+    <tableColumn id="26" xr3:uid="{BE249C9E-41CD-4B49-97DA-A0B62966DEFF}" name="COMMENTS"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium28" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheets">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Sheets">
   <a:themeElements>
     <a:clrScheme name="Sheets">
       <a:dk1>
@@ -351,17 +451,27 @@
       </a:bgFillStyleLst>
     </a:fmtScheme>
   </a:themeElements>
+  <a:objectDefaults/>
+  <a:extraClrSchemeLst/>
 </a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
-  <sheetFormatPr customHeight="1" defaultColWidth="12.63" defaultRowHeight="15.75"/>
+  <dimension ref="A1:Z4"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="12.5703125" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="1" max="1" width="23.7109375" customWidth="1"/>
+    <col min="26" max="26" width="37.85546875" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1">
+    <row r="1" spans="1:26" x14ac:dyDescent="0.2">
+      <c r="A1" t="s">
+        <v>32</v>
+      </c>
       <c r="B1" s="1" t="s">
         <v>0</v>
       </c>
@@ -438,22 +548,100 @@
         <v>24</v>
       </c>
     </row>
-    <row r="2">
+    <row r="2" spans="1:26" x14ac:dyDescent="0.2">
       <c r="A2" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="B2" t="s">
+        <v>28</v>
+      </c>
+      <c r="C2" t="s">
+        <v>28</v>
+      </c>
+      <c r="D2" t="s">
+        <v>28</v>
+      </c>
+      <c r="E2" t="s">
+        <v>28</v>
+      </c>
+      <c r="F2" t="s">
+        <v>28</v>
+      </c>
+      <c r="G2" t="s">
+        <v>28</v>
+      </c>
+      <c r="H2" t="s">
+        <v>27</v>
+      </c>
+      <c r="I2" t="s">
+        <v>27</v>
+      </c>
+      <c r="J2" t="s">
+        <v>27</v>
+      </c>
+      <c r="K2" t="s">
+        <v>29</v>
+      </c>
+      <c r="L2" t="s">
+        <v>29</v>
+      </c>
+      <c r="M2" t="s">
+        <v>27</v>
+      </c>
+      <c r="N2" t="s">
+        <v>27</v>
+      </c>
+      <c r="O2" t="s">
+        <v>29</v>
+      </c>
+      <c r="P2" t="s">
+        <v>29</v>
+      </c>
+      <c r="Q2" t="s">
+        <v>27</v>
+      </c>
+      <c r="R2" t="s">
+        <v>29</v>
+      </c>
+      <c r="S2" t="s">
+        <v>28</v>
+      </c>
+      <c r="T2" t="s">
+        <v>30</v>
+      </c>
+      <c r="U2" t="s">
+        <v>27</v>
+      </c>
+      <c r="V2" t="s">
+        <v>28</v>
+      </c>
+      <c r="W2" t="s">
+        <v>29</v>
+      </c>
+      <c r="X2" t="s">
+        <v>30</v>
+      </c>
+      <c r="Y2" t="s">
+        <v>28</v>
+      </c>
+      <c r="Z2" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="3" spans="1:26" x14ac:dyDescent="0.2">
+      <c r="A3" s="1" t="s">
         <v>25</v>
       </c>
     </row>
-    <row r="3">
-      <c r="A3" s="1" t="s">
+    <row r="4" spans="1:26" x14ac:dyDescent="0.2">
+      <c r="A4" s="1" t="s">
         <v>26</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="1" t="s">
-        <v>27</v>
       </c>
     </row>
   </sheetData>
-  <drawing r:id="rId1"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <tableParts count="1">
+    <tablePart r:id="rId1"/>
+  </tableParts>
 </worksheet>
 </file>
</xml_diff>